<commit_message>
Add KAKERO principles check and data v0.1
</commit_message>
<xml_diff>
--- a/kakero-wbs/KAKERO_WBS.xlsx
+++ b/kakero-wbs/KAKERO_WBS.xlsx
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryTable" displayName="SummaryTable" ref="A4:B17" headerRowCount="1">
-  <autoFilter ref="A4:B17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SummaryTable" displayName="SummaryTable" ref="A4:B16" headerRowCount="1">
+  <autoFilter ref="A4:B16"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Item"/>
     <tableColumn id="2" name="Content"/>
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="WBSTable" displayName="WBSTable" ref="A4:H46" headerRowCount="1">
-  <autoFilter ref="A4:H46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="WBSTable" displayName="WBSTable" ref="A4:H48" headerRowCount="1">
+  <autoFilter ref="A4:H48"/>
   <tableColumns count="8">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Phase"/>
@@ -206,8 +206,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="OPENQUESTIONSTable" displayName="OPENQUESTIONSTable" ref="A4:F25" headerRowCount="1">
-  <autoFilter ref="A4:F25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="OPENQUESTIONSTable" displayName="OPENQUESTIONSTable" ref="A4:F27" headerRowCount="1">
+  <autoFilter ref="A4:F27"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="ID"/>
@@ -221,8 +221,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DECISIONLOGTable" displayName="DECISIONLOGTable" ref="A4:E20" headerRowCount="1">
-  <autoFilter ref="A4:E20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DECISIONLOGTable" displayName="DECISIONLOGTable" ref="A4:E23" headerRowCount="1">
+  <autoFilter ref="A4:E23"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="日付"/>
@@ -235,8 +235,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="REJECTEDIDEASTable" displayName="REJECTEDIDEASTable" ref="A4:E21" headerRowCount="1">
-  <autoFilter ref="A4:E21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="REJECTEDIDEASTable" displayName="REJECTEDIDEASTable" ref="A4:E22" headerRowCount="1">
+  <autoFilter ref="A4:E22"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="案"/>
@@ -249,8 +249,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PRINCIPLESTable" displayName="PRINCIPLESTable" ref="A4:B11" headerRowCount="1">
-  <autoFilter ref="A4:B11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PRINCIPLESTable" displayName="PRINCIPLESTable" ref="A4:B12" headerRowCount="1">
+  <autoFilter ref="A4:B12"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Principle"/>
     <tableColumn id="2" name="Content"/>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Excel view. OPEN_QUESTIONS holds undecided items; PRINCIPLES holds review rules.</t>
+          <t>Excel view. Open items remain open; prices and business decisions are not silently decided.</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Required docs</t>
+          <t>New outputs</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>WBS.md / OPEN_QUESTIONS.md / DECISION_LOG.md / KAKERO_PRINCIPLES.md</t>
+          <t>KAKERO_PRINCIPLES_CHECK.html / GOODHART_REVIEW_CHECKLIST.md / PLAY_LAYER_POC_CANDIDATES.md / KAKERO_DATA_v0.1.md / sample JSON files</t>
         </is>
       </c>
     </row>
@@ -613,14 +613,14 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Entry and retention engine are play. Essential payoff is that life becomes a board.</t>
+          <t>Entry and retention engine are play. Essential payoff is life becoming a board.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Goodhart avoidance</t>
+          <t>Goodhart</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -632,94 +632,82 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Pricing principle</t>
+          <t>Data v0.1</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Barbell: 0 yen and 3000 yen. No weak middle price ladder.</t>
+          <t>OKF-like custom JSON with board / nodes / edges / health_map / memory_items / metadata</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Scale</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>52-84 person-days, roughly 4.5-7 months at side-project pace</t>
-        </is>
-      </c>
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Phase scale</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Phase scale</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
+          <t>Phase 0-2</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>9-14人日 / 3-5週間 / データ骨格とHaikuカード化PoC</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Phase 0-2</t>
+          <t>Phase 3-4</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>9-14人日 / 3-5週間 / データ骨格とHaikuカード化PoC</t>
+          <t>15-24人日 / 5-8週間 / コンパス/けんこうマップ反映PoC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Phase 3-4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>15-24人日 / 5-8週間 / コンパス/けんこうマップ反映PoC</t>
+          <t>22-38人日 / 7-12週間 / 商品 walking skeleton、遊びレイヤーPoC、原則確認ページ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>22-38人日 / 7-12週間 / 商品 walking skeleton、遊びレイヤーPoC、原則確認ページ</t>
+          <t>5-8人日 / 1-2週間 / 技術GO / 体験GO / 事業GO 判定</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>合計</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>5-8人日 / 1-2週間 / 技術GO / 体験GO / 事業GO 判定</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>52-84人日 / 4.5-7か月目安 / 最低限遊べる商品状態とGO判定</t>
         </is>
@@ -743,14 +731,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -1067,91 +1055,91 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>データの骨</t>
+          <t>文書・台帳整備</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>KAKERO内部スキーマ v0.1 を定義する</t>
+          <t>Goodhart回避レビュー観点をチェックリスト化する</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>KAKERO_DATA_v0.1.md</t>
+          <t>GOODHART_REVIEW_CHECKLIST.md</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>nodes, edges, health_map, memory_items, metadata の役割が定義されている</t>
+          <t>ゲーム要素追加時に人生マップの正直さを壊していないか確認できる</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>データの骨</t>
+          <t>文書・台帳整備</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>サンプル盤面データを作る</t>
+          <t>遊びレイヤーPoC候補を2-3個に絞る</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>sample_board.json</t>
+          <t>PLAY_LAYER_POC_CANDIDATES.md</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.6, 0.7</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>10カード前後、サブカード、小タスク、依存、状態、記憶項目、けんこうマップが入っている</t>
+          <t>突発イベント/隠し報酬、変な称号、きこうか君変化の扱いと優先度が整理されている</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0.5-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1166,34 +1154,34 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Haiku出力サンプルを作る</t>
+          <t>KAKERO内部スキーマ v0.1 を定義する</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>sample_haiku_output.json</t>
+          <t>KAKERO_DATA_v0.1.md</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.4, 0.6</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>6フィールド出力と内部スキーマ変換後の形が対応している</t>
+          <t>nodes, edges, health_map, memory_items, metadata の役割が定義されている</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>0.5-1</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1208,12 +1196,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>盤面をAIへ渡す入力形式を決める</t>
+          <t>サンプル盤面データを作る</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>AI入力ペイロード仕様</t>
+          <t>sample_board.json</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1223,7 +1211,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>会話ログなしで、既存カード・マップ値・記憶項目を渡せる</t>
+          <t>10カード前後、サブカード、小タスク、依存、状態、記憶項目、けんこうマップが入っている</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1235,12 +1223,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Haikuカード化PoC</t>
+          <t>データの骨</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1250,39 +1238,39 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>API中継の最小構成を作る</t>
+          <t>Haiku出力サンプルを作る</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Haiku中継PoC</t>
+          <t>sample_haiku_output.json</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>1発話1コール、履歴なし、temperature低めで呼べる</t>
+          <t>6フィールド出力と内部スキーマ変換後の形が対応している</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0.5-1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Haikuカード化PoC</t>
+          <t>データの骨</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1292,34 +1280,34 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>6フィールドJSON出力を検証する</t>
+          <t>盤面をAIへ渡す入力形式を決める</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>カード化テスト結果</t>
+          <t>AI入力ペイロード仕様</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>願望系テスト発話が card/subcards/tasks/premises/dependencies/success に分解される</t>
+          <t>会話ログなしで、既存カード・マップ値・記憶項目を渡せる</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1334,34 +1322,34 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>脱線拒否を検証する</t>
+          <t>API中継の最小構成を作る</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>脱線テスト結果</t>
+          <t>Haiku中継PoC</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>雑談・天気・愚痴・きこうか君への話しかけを イマソノハナシヲシテマセン で弾ける</t>
+          <t>1発話1コール、履歴なし、temperature低めで呼べる</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>0.5-1</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1376,12 +1364,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>複数願望混在入力を検証する</t>
+          <t>6フィールドJSON出力を検証する</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>混在入力テスト結果</t>
+          <t>カード化テスト結果</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1391,19 +1379,19 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>「金欲しい、モテたい、引っ越したい」を中心カード+関連要素へ畳める</t>
+          <t>願望系テスト発話が card/subcards/tasks/premises/dependencies/success に分解される</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1418,34 +1406,34 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>内部スキーマへの変換を検証する</t>
+          <t>脱線拒否を検証する</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>変換PoC</t>
+          <t>脱線テスト結果</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>2.2, 2.3, 2.4</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Haiku出力が nodes/edges/metadata に破綻なく入る</t>
+          <t>雑談・天気・愚痴・きこうか君への話しかけを イマソノハナシヲシテマセン で弾ける</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0.5-1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1460,22 +1448,22 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Haiku採用/上位モデル再判定を行う</t>
+          <t>複数願望混在入力を検証する</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>技術判定メモ</t>
+          <t>混在入力テスト結果</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>2.2, 2.3, 2.4, 2.5</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Haiku継続、プロンプト修正、Sonnet再検証のいずれかが判断できる</t>
+          <t>「金欲しい、モテたい、引っ越したい」を中心カード+関連要素へ畳める</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1487,12 +1475,12 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>人生コンパス反映PoC</t>
+          <t>Haikuカード化PoC</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1502,22 +1490,22 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>既存 compass-board ソースを調査する</t>
+          <t>内部スキーマへの変換を検証する</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>調査メモ</t>
+          <t>変換PoC</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>2.2, 2.3, 2.4</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>技術構成、表示構造、流用可否、改修ポイントが分かる</t>
+          <t>Haiku出力が nodes/edges/metadata に破綻なく入る</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1529,12 +1517,12 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>人生コンパス反映PoC</t>
+          <t>Haikuカード化PoC</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1544,34 +1532,34 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>KAKEROデータをコンパス表示へ流し込む</t>
+          <t>Haiku採用/上位モデル再判定を行う</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>コンパス反映PoC</t>
+          <t>技術判定メモ</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>1.2, 3.1</t>
+          <t>2.2, 2.3, 2.4, 2.5</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>sample_board のカードが画面に表示される</t>
+          <t>Haiku継続、プロンプト修正、Sonnet再検証のいずれかが判断できる</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1586,22 +1574,22 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>10カード表示を検証する</t>
+          <t>既存 compass-board ソースを調査する</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>10カード表示PoC</t>
+          <t>調査メモ</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>10個前後並べても「人生コンパスっぽい」俯瞰が崩れない</t>
+          <t>技術構成、表示構造、流用可否、改修ポイントが分かる</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1613,7 +1601,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1628,34 +1616,34 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>状態表示ルールを反映する</t>
+          <t>KAKEROデータをコンパス表示へ流し込む</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>状態表示PoC</t>
+          <t>コンパス反映PoC</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>1.2, 3.1</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>未着手/実行中/完了/大達成/未解放/待機/メモあり等を識別できる</t>
+          <t>sample_board のカードが画面に表示される</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1670,12 +1658,12 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>手編集PoCを作る</t>
+          <t>10カード表示を検証する</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>編集PoC</t>
+          <t>10カード表示PoC</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1685,19 +1673,19 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>カードの編集、移動、削除、状態変更ができる</t>
+          <t>10個前後並べても「人生コンパスっぽい」俯瞰が崩れない</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1712,22 +1700,22 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>編集結果を盤面に保存/復元する</t>
+          <t>状態表示ルールを反映する</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>保存復元PoC</t>
+          <t>状態表示PoC</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>リロード後も編集結果が残る。保存方式は作りやすさ優先で仮置き</t>
+          <t>未着手/実行中/完了/大達成/未解放/待機/メモあり等を識別できる</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1739,12 +1727,12 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>けんこうマップ反映PoC</t>
+          <t>人生コンパス反映PoC</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1754,39 +1742,39 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>けんこうマップの最小データ構造を定義する</t>
+          <t>手編集PoCを作る</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>health_map仕様</t>
+          <t>編集PoC</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>生活/仕事/心身/金/家族/余白などの反映先が定義されている</t>
+          <t>カードの編集、移動、削除、状態変更ができる</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>けんこうマップ反映PoC</t>
+          <t>人生コンパス反映PoC</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1796,34 +1784,34 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>カードからけんこうマップへ反映する</t>
+          <t>編集結果を盤面に保存/復元する</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>けんこう反映PoC</t>
+          <t>保存復元PoC</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>2.5, 4.1</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>カード追加でマップ項目・総合点・今月モード候補が変化する</t>
+          <t>リロード後も編集結果が残る。保存方式は作りやすさ優先で仮置き</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1838,34 +1826,34 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>単なるToDo化していないか検証する</t>
+          <t>けんこうマップの最小データ構造を定義する</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>体験レビュー結果</t>
+          <t>health_map仕様</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>カードとマップの関係が意味ある状態変化として見える</t>
+          <t>生活/仕事/心身/金/家族/余白などの反映先が定義されている</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1875,86 +1863,86 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>PoC必要</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>初期自動反映精度を調整する</t>
+          <t>カードからけんこうマップへ反映する</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>調整方針メモ</t>
+          <t>けんこう反映PoC</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>4.2, OPEN_QUESTIONS.md</t>
+          <t>2.5, 4.1</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>自動反映の深さを「WSで必要な最低限」に抑えられている</t>
+          <t>カード追加でマップ項目・総合点・今月モード候補が変化する</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>商品walking skeleton</t>
+          <t>けんこうマップ反映PoC</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>決定済み</t>
+          <t>PoC必要</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>LP/入口を作る</t>
+          <t>単なるToDo化していないか検証する</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>入口画面</t>
+          <t>体験レビュー結果</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>KAKEROが何か、初回体験へ進めることが分かる</t>
+          <t>カードとマップの関係が意味ある状態変化として見える</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>商品walking skeleton</t>
+          <t>けんこうマップ反映PoC</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1964,34 +1952,34 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>LPコピーを仮置きする</t>
+          <t>初期自動反映精度を調整する</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>仮コピー</t>
+          <t>調整方針メモ</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>5.1, OPEN_QUESTIONS.md</t>
+          <t>4.2, OPEN_QUESTIONS.md</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>最終コピーを確定せず、検証用文言で入口が成立する</t>
+          <t>自動反映の深さを「WSで必要な最低限」に抑えられている</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>0.5-1</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -2006,34 +1994,34 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>プラン/価格ページを作る</t>
+          <t>LP/入口を作る</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>プラン/価格ページ</t>
+          <t>入口画面</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>本番決済なしで、有料エンジンの価値と無料範囲が説明されている</t>
+          <t>KAKEROが何か、初回体験へ進めることが分かる</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2043,39 +2031,39 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>決定済み</t>
+          <t>未確定</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>きこうか君チュートリアルを作る</t>
+          <t>LPコピーを仮置きする</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>チュートリアル導線</t>
+          <t>仮コピー</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>2.5, 5.1</t>
+          <t>5.1, OPEN_QUESTIONS.md</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>「ヤア、ワタシガキコウカクンデス」から願望入力へ進める</t>
+          <t>最終コピーを確定せず、検証用文言で入口が成立する</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>0.5-1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2085,39 +2073,39 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>10カード登録体験を通す</t>
+          <t>プラン/価格ページを作る</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>初回登録フロー</t>
+          <t>プラン/価格ページ</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>5.4, 3.3, 4.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>初回体験で5-10カードを登録し、盤面化できる</t>
+          <t>本番決済なしで、有料エンジンの価値と無料範囲が説明されている</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2132,22 +2120,22 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>覚えてほしいことリストを作る</t>
+          <t>きこうか君チュートリアルを作る</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>memory_items UI</t>
+          <t>チュートリアル導線</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>1.1, 5.4</t>
+          <t>2.5, 5.1</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>10-20個程度の記憶項目を追加/編集でき、AI入力に含められる</t>
+          <t>「ヤア、ワタシガキコウカクンデス」から願望入力へ進める</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2159,7 +2147,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2174,34 +2162,34 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>次回きこうか君が盤面を理解するループを作る</t>
+          <t>10カード登録体験を通す</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>盤面理解PoC</t>
+          <t>初回登録フロー</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>1.4, 3.6, 5.6</t>
+          <t>5.4, 3.3, 4.2</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>会話履歴なしで、既存盤面を踏まえたカード化/修正ができる</t>
+          <t>初回体験で5-10カードを登録し、盤面化できる</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-5</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2211,27 +2199,27 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>今日の9タスク導線を仮実装する</t>
+          <t>覚えてほしいことリストを作る</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>今日タスク仮画面</t>
+          <t>memory_items UI</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>3.6, 4.2, OPEN_QUESTIONS.md</t>
+          <t>1.1, 5.4</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>自動生成ロジック未確定のため、仮選定または手動選択で体験確認できる</t>
+          <t>10-20個程度の記憶項目を追加/編集でき、AI入力に含められる</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2243,7 +2231,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -2258,34 +2246,34 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>遊びレイヤーPoCを作る</t>
+          <t>次回きこうか君が盤面を理解するループを作る</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>遊びレイヤーPoC</t>
+          <t>盤面理解PoC</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>5.4, 5.5, KAKERO_PRINCIPLES.md</t>
+          <t>1.4, 3.6, 5.6</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>かわいい、楽しい、変な称号、育て要素、突発イベント、隠し要素のうち最低2-3要素を体験として試せる</t>
+          <t>会話履歴なしで、既存盤面を踏まえたカード化/修正ができる</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2295,27 +2283,27 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>未確定</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>予期しない報酬PoCを作る</t>
+          <t>今日の9タスク導線を仮実装する</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>突発イベント/隠し報酬PoC</t>
+          <t>今日タスク仮画面</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>5.9, OPEN_QUESTIONS.md</t>
+          <t>3.6, 4.2, OPEN_QUESTIONS.md</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>卵に固定せず、無料ユーザー向け試食体験や隠し報酬が毎日開く理由になるか検証できる</t>
+          <t>自動生成ロジック未確定のため、仮選定または手動選択で体験確認できる</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2327,7 +2315,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>5.11</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -2337,39 +2325,39 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>決定済み</t>
+          <t>PoC必要</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>原則確認ページ案を作る</t>
+          <t>遊びレイヤーPoCを作る</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>KAKERO_PRINCIPLES_CHECK.html</t>
+          <t>遊びレイヤーPoC</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.8, 5.4, 5.5, KAKERO_PRINCIPLES.md</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>スマホで短く「これはKAKEROか？」を確認でき、実装/レビュー時に長文原則へ戻れる</t>
+          <t>かわいい、楽しい、変な称号、育て要素、突発イベント、隠し要素のうち最低2-3要素を体験として試せる</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>3-5</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>5.10</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2379,123 +2367,123 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>決定済み</t>
+          <t>PoC必要</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>WS統合テストを行う</t>
+          <t>予期しない報酬PoCを作る</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>WSテスト結果</t>
+          <t>突発イベント/隠し報酬PoC</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>5.1-5.11</t>
+          <t>0.7, 0.8, 5.9, OPEN_QUESTIONS.md</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>入口 -&gt; チュートリアル -&gt; カード化 -&gt; コンパス/けんこう反映 -&gt; 手編集 -&gt; 遊びレイヤー -&gt; 再読込 が通る</t>
+          <t>卵に固定せず、無料ユーザー向け試食体験や隠し報酬が毎日開く理由になるか検証できる</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>2-4</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.11</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>GO判定</t>
+          <t>商品walking skeleton</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>技術GOを判定する</t>
+          <t>原則確認ページ案を作る</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>技術GO判定メモ</t>
+          <t>KAKERO_PRINCIPLES_CHECK.html</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>0.6, 0.7</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Haiku、盤面、編集、保存、けんこう反映が通る/通らないを判断できる</t>
+          <t>スマホで短く「これはKAKEROか？」を確認でき、実装/レビュー時に長文原則へ戻れる</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.12</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>GO判定</t>
+          <t>商品walking skeleton</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>PoC必要</t>
+          <t>決定済み</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>体験GOを判定する</t>
+          <t>WS統合テストを行う</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>体験GO判定メモ</t>
+          <t>WSテスト結果</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>5.1-5.11</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>10カード前後で「こうなるのね」が出ることに加え、遊びレイヤーが毎日開く理由になるか判断できる</t>
+          <t>入口 -&gt; チュートリアル -&gt; カード化 -&gt; コンパス/けんこう反映 -&gt; 手編集 -&gt; 遊びレイヤー -&gt; 再読込 が通る</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2505,72 +2493,156 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>PoC必要</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>事業GOを判定する</t>
+          <t>技術GOを判定する</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>事業GO判定メモ</t>
+          <t>技術GO判定メモ</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>5.1, 5.3, 5.5, 5.9, OPEN_QUESTIONS.md</t>
+          <t>5.12</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>ICP/価格/継続/集客/粗利の未決を明示したうえで次判断に進める</t>
+          <t>Haiku、盤面、編集、保存、けんこう反映が通る/通らないを判断できる</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>GO判定</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>PoC必要</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>体験GOを判定する</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>体験GO判定メモ</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>5.12</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>10カード前後で「こうなるのね」が出ることに加え、遊びレイヤーが毎日開く理由になるか判断できる</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>GO判定</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>未確定</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>事業GOを判定する</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>事業GO判定メモ</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>5.1, 5.3, 5.5, 5.9, OPEN_QUESTIONS.md</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>ICP/価格/継続/集客/粗利の未決を明示したうえで次判断に進める</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>GO判定</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>決定済み</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>次フェーズ計画を作る</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>次フェーズWBS</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>6.1, 6.2, 6.3</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>本実装へ進む/PoC追加/事業検証優先/保留のいずれかが明確</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2594,14 +2666,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3038,32 +3110,32 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>データ・保存</t>
+          <t>体験・仕様</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>OQ-201</t>
+          <t>OQ-108</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>保存方式の本決定</t>
+          <t>遊びレイヤーPoCの実装順</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>初期は作りやすさ優先</t>
+          <t>候補整理は完了。実装確定ではない</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>PoCでは仮保存。将来は端末ローカル保存/移行を有力候補</t>
+          <t>PLAY_LAYER_POC_CANDIDATES.md を元に、walking skeletonへ入れる最小PoCを選ぶ</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>本実装前</t>
+          <t>商品WS設計前</t>
         </is>
       </c>
     </row>
@@ -3075,27 +3147,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>OQ-202</t>
+          <t>OQ-201</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>スマホ移行/エクスポート/インポート</t>
+          <t>保存方式の本決定</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>将来候補</t>
+          <t>初期は作りやすさ優先</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>walking skeleton外</t>
+          <t>PoCでは仮保存。将来は端末ローカル保存/移行を有力候補</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>保存方式本決定後</t>
+          <t>本実装前</t>
         </is>
       </c>
     </row>
@@ -3107,27 +3179,27 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>OQ-203</t>
+          <t>OQ-202</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Cloudflare側に盤面保存を持たせるか</t>
+          <t>スマホ移行/エクスポート/インポート</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>将来候補</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>初期PoCでは強く前提化しない</t>
+          <t>walking skeleton外</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>ログイン/同期検討時</t>
+          <t>保存方式本決定後</t>
         </is>
       </c>
     </row>
@@ -3139,91 +3211,91 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>OQ-204</t>
+          <t>OQ-203</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>既存 compass-board の実際のソース構成</t>
+          <t>Cloudflare側に盤面保存を持たせるか</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>ソースあり前提</t>
+          <t>未確定</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Phase 3.1で調査</t>
+          <t>初期PoCでは強く前提化しない</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>コンパス反映PoC前</t>
+          <t>ログイン/同期検討時</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>事業GO</t>
+          <t>データ・保存</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>OQ-301</t>
+          <t>OQ-204</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>ICPの最終定義</t>
+          <t>既存 compass-board の実際のソース構成</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>仮説あり</t>
+          <t>ソースあり前提</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>事業GO判定で明文化</t>
+          <t>Phase 3.1で調査</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>事業検証開始前</t>
+          <t>コンパス反映PoC前</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>事業GO</t>
+          <t>データ・保存</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>OQ-302</t>
+          <t>OQ-205</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>事業GOの数値基準</t>
+          <t>v0.1データ構造の保存方式</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>仮説あり</t>
+          <t>構造定義とサンプルは作成済み</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Phase 6で仮基準を置き、未検証なら未決扱い</t>
+          <t>初期は作りやすさ優先。保存先の本決定はしない</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>GO判定時</t>
+          <t>本実装前</t>
         </is>
       </c>
     </row>
@@ -3235,27 +3307,27 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>OQ-303</t>
+          <t>OQ-301</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>初期獲得チャネル</t>
+          <t>ICPの最終定義</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>仮説あり</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>まず手売り/少人数検証寄りで仮置き</t>
+          <t>事業GO判定で明文化</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>事業GO判定前</t>
+          <t>事業検証開始前</t>
         </is>
       </c>
     </row>
@@ -3267,27 +3339,27 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>OQ-304</t>
+          <t>OQ-302</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>月額3000円に対する支払い意思</t>
+          <t>事業GOの数値基準</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>仮説あり</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>価格ページ/聞き取りで検証</t>
+          <t>Phase 6で仮基準を置き、未検証なら未決扱い</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Revenue Validation時</t>
+          <t>GO判定時</t>
         </is>
       </c>
     </row>
@@ -3299,25 +3371,89 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>OQ-303</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>初期獲得チャネル</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>未確定</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>まず手売り/少人数検証寄りで仮置き</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>事業GO判定前</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>事業GO</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>OQ-304</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>月額3000円に対する支払い意思</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>価格ページ/聞き取りで検証</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Revenue Validation時</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>事業GO</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
           <t>OQ-305</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>AI原価の許容ライン</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>仮説あり</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Unit Economicsで検証</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>有料化前</t>
         </is>
@@ -3341,14 +3477,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3821,6 +3957,87 @@
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>突発イベント/隠し報酬/無料ユーザー向け試食体験のPoC候補にする</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>DL-017</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>原則確認ページをレビュー補助成果物として作る</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>長文原則は実装・レビュー時に読まれなくなる可能性がある</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>KAKERO_PRINCIPLES_CHECK.html でスマホ確認できるようにする</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>DL-018</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>KAKERO内部データ v0.1 はOKF風の自前JSONで開始する</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>正式OKF準拠は不要だが、nodes/edges的な構造は後のAI変換と拡張に効く</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>KAKERO_DATA_v0.1.md、sample_board.json、sample_haiku_output.json を初期成果物にする</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>DL-019</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>遊びレイヤーPoC候補は2-3個に絞って検証する</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>最初から遊び本実装を広げると発散する</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>突発イベント/隠し報酬、変な称号、きこうか君変化を候補にする</t>
         </is>
       </c>
     </row>
@@ -3842,14 +4059,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4349,6 +4566,33 @@
       <c r="E21" s="4" t="inlineStr">
         <is>
           <t>3000円転換が重すぎると検証された後</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>RI-018</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>遊びレイヤーの一括本実装</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>後回し</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>継続エンジンとして重要だが、最初から作り込むとwalking skeletonが肥大化する</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>体験PoCで刺さる要素が見えた後</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4508,6 +4752,20 @@
 - これはゲーム報酬のために人生マップをハックさせないか
 - これは0円/3000円のバーベルを濁していないか
 - これは人生データを人質にしていないか</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>8. 短い確認ページ</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>実装・レビュー時は、長文原則だけに頼らない。
+スマホで短く確認できる `KAKERO_PRINCIPLES_CHECK.html` を併用する。
+目的は、レビュー時に「これはKAKEROか？」をその場で確認すること。</t>
         </is>
       </c>
     </row>

</xml_diff>